<commit_message>
Added API of the newly launched index
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AABF882-ED42-41BA-9CA4-1E0367142D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF47F09-CA66-42B0-A1C6-AC0B3243338C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="broad" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="194">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -616,6 +616,9 @@
   </si>
   <si>
     <t>NIFTY500 GROWTH 50</t>
+  </si>
+  <si>
+    <t>NIFTY AI CATALYSTS</t>
   </si>
 </sst>
 </file>
@@ -1892,7 +1895,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{466D5EDC-7427-4A89-B90E-E56187B74B61}">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.6640625" style="1" customWidth="1"/>
@@ -2612,6 +2615,20 @@
       </c>
       <c r="D51" t="s">
         <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B52" s="3">
+        <v>45471</v>
+      </c>
+      <c r="C52">
+        <v>1000</v>
+      </c>
+      <c r="D52" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>